<commit_message>
determining the actual rpm of the fan
</commit_message>
<xml_diff>
--- a/Fan Speed Data.xlsx
+++ b/Fan Speed Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://purdue0-my.sharepoint.com/personal/knigh152_purdue_edu/Documents/2k7/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ian\vertical-farm-automation-summer-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0C7C9D0F-1DE8-4204-A6EE-C3B127D2BEFD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C6AF2D-60AD-4E34-AF3B-E0D7A9406AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{9287F51C-2EFF-4DAB-AE9E-BB1DC553013A}"/>
+    <workbookView xWindow="-96" yWindow="6840" windowWidth="11712" windowHeight="6936" xr2:uid="{9287F51C-2EFF-4DAB-AE9E-BB1DC553013A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,6 +36,47 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+  <si>
+    <t>?</t>
+  </si>
+  <si>
+    <t>YES</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>Max</t>
+  </si>
+  <si>
+    <t>very low</t>
+  </si>
+  <si>
+    <t>duty</t>
+  </si>
+  <si>
+    <t>start reliably</t>
+  </si>
+  <si>
+    <t>estimated speed</t>
+  </si>
+  <si>
+    <t>Vfg</t>
+  </si>
+  <si>
+    <t>Ic</t>
+  </si>
+  <si>
+    <t>R (must &gt;=)</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -69,8 +110,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -405,14 +452,118 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FACF1BAE-EDBA-4EFB-A6D7-5115C050F8EB}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F1" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="1">
+        <v>0.1</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>15</v>
+      </c>
+      <c r="F2">
+        <f>5*0.001</f>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G2">
+        <f>E2/F2</f>
+        <v>3000</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="1">
+        <v>0.5</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="1">
+        <v>1</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="97678919-6b7f-4801-8308-74906889bf8c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101001D59A680A57AA148B60D2183F26FBF78" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="8fa533ab1ceddead104f9c52f8263840">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="97678919-6b7f-4801-8308-74906889bf8c" xmlns:ns4="4a3de536-389c-4315-8a87-e926c024be71" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9be2744d9fb7d894ef4dc43ef325cb5e" ns3:_="" ns4:_="">
     <xsd:import namespace="97678919-6b7f-4801-8308-74906889bf8c"/>
@@ -651,24 +802,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="97678919-6b7f-4801-8308-74906889bf8c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F462480-397F-4966-A075-1EC130895638}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="4a3de536-389c-4315-8a87-e926c024be71"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="97678919-6b7f-4801-8308-74906889bf8c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55B6BB06-BC2D-478D-A136-A7CF35C12E1D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{58D36F72-B7F5-448F-9194-E4BA036C20D2}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -685,29 +844,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55B6BB06-BC2D-478D-A136-A7CF35C12E1D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F462480-397F-4966-A075-1EC130895638}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="4a3de536-389c-4315-8a87-e926c024be71"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="97678919-6b7f-4801-8308-74906889bf8c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
PID control loop for fan speed control is working
</commit_message>
<xml_diff>
--- a/Fan Speed Data.xlsx
+++ b/Fan Speed Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ian\vertical-farm-automation-summer-2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C6AF2D-60AD-4E34-AF3B-E0D7A9406AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9204E511-3987-4A38-A11F-CAEA2F9FD6B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="6840" windowWidth="11712" windowHeight="6936" xr2:uid="{9287F51C-2EFF-4DAB-AE9E-BB1DC553013A}"/>
+    <workbookView xWindow="11424" yWindow="6840" windowWidth="11712" windowHeight="6936" xr2:uid="{9287F51C-2EFF-4DAB-AE9E-BB1DC553013A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="21">
   <si>
     <t>?</t>
   </si>
@@ -75,6 +75,33 @@
   </si>
   <si>
     <t>R (must &gt;=)</t>
+  </si>
+  <si>
+    <t>PID params</t>
+  </si>
+  <si>
+    <t>ki</t>
+  </si>
+  <si>
+    <t>kd</t>
+  </si>
+  <si>
+    <t>test run #</t>
+  </si>
+  <si>
+    <t>target speed (RPM)</t>
+  </si>
+  <si>
+    <t>sample rate (s)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kp </t>
+  </si>
+  <si>
+    <t>taskkill /F /IM python.exe</t>
+  </si>
+  <si>
+    <t>cd C:\Users\Ian\vertical-farm-automation-summer-2026</t>
   </si>
 </sst>
 </file>
@@ -452,10 +479,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FACF1BAE-EDBA-4EFB-A6D7-5115C050F8EB}">
-  <dimension ref="A1:G6"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="3" max="3" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.77734375" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -475,7 +506,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1">
         <v>0.1</v>
       </c>
@@ -497,7 +528,7 @@
         <v>3000</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1">
         <v>0.2</v>
       </c>
@@ -508,7 +539,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A4" s="1">
         <v>0.3</v>
       </c>
@@ -519,7 +550,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1">
         <v>0.5</v>
       </c>
@@ -529,8 +560,11 @@
       <c r="C5" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="H5" t="s">
+        <v>19</v>
+      </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1">
         <v>1</v>
       </c>
@@ -539,6 +573,40 @@
       </c>
       <c r="C6" s="2" t="s">
         <v>4</v>
+      </c>
+      <c r="H6" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E8" t="s">
+        <v>18</v>
+      </c>
+      <c r="F8" t="s">
+        <v>13</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9">
+        <v>4680</v>
       </c>
     </row>
   </sheetData>
@@ -547,20 +615,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="97678919-6b7f-4801-8308-74906889bf8c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="97678919-6b7f-4801-8308-74906889bf8c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -803,6 +871,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55B6BB06-BC2D-478D-A136-A7CF35C12E1D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4F462480-397F-4966-A075-1EC130895638}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -815,14 +891,6 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="97678919-6b7f-4801-8308-74906889bf8c"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55B6BB06-BC2D-478D-A136-A7CF35C12E1D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>